<commit_message>
Distribution SAQ — 2026-06-08
</commit_message>
<xml_diff>
--- a/Distribution_SAQ_20260608.xlsx
+++ b/Distribution_SAQ_20260608.xlsx
@@ -18,7 +18,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="5">
+  <fonts count="7">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -45,8 +45,18 @@
     <font>
       <name val="Arial"/>
       <b val="1"/>
+      <color rgb="0000703C"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
       <color rgb="00C00000"/>
       <sz val="10"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <sz val="9"/>
     </font>
   </fonts>
   <fills count="5">
@@ -84,7 +94,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -107,9 +117,10 @@
     <xf numFmtId="0" fontId="3" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -531,18 +542,14 @@
         </is>
       </c>
       <c r="C3" s="5" t="n">
-        <v>0</v>
+        <v>264</v>
       </c>
       <c r="D3" s="4" t="inlineStr">
         <is>
-          <t>erreur_api</t>
-        </is>
-      </c>
-      <c r="E3" s="4" t="inlineStr">
-        <is>
-          <t>400 Client Error: Bad Request for url: https://www.saq.com/en/store/locator/ajaxlist/context/product/id/417396?loaded=0&amp;latitude=45.5088&amp;longitude=-73.5540</t>
-        </is>
-      </c>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="E3" s="4" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" s="6" t="inlineStr">
@@ -583,7 +590,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F1"/>
+  <dimension ref="A1:F11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -626,6 +633,306 @@
         </is>
       </c>
     </row>
+    <row r="2">
+      <c r="A2" s="9" t="inlineStr">
+        <is>
+          <t>15544570</t>
+        </is>
+      </c>
+      <c r="B2" s="9" t="inlineStr">
+        <is>
+          <t>Beach Day Every Day Vodka Frozen Berries</t>
+        </is>
+      </c>
+      <c r="C2" s="9" t="inlineStr">
+        <is>
+          <t>De Maisonneuve - City Councillors</t>
+        </is>
+      </c>
+      <c r="D2" s="9" t="inlineStr">
+        <is>
+          <t>SAQ Sélection</t>
+        </is>
+      </c>
+      <c r="E2" s="9" t="inlineStr">
+        <is>
+          <t>Montréal</t>
+        </is>
+      </c>
+      <c r="F2" s="9" t="n">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="9" t="inlineStr">
+        <is>
+          <t>15544570</t>
+        </is>
+      </c>
+      <c r="B3" s="9" t="inlineStr">
+        <is>
+          <t>Beach Day Every Day Vodka Frozen Berries</t>
+        </is>
+      </c>
+      <c r="C3" s="9" t="inlineStr">
+        <is>
+          <t>La Cité - Les Galeries du Parc</t>
+        </is>
+      </c>
+      <c r="D3" s="9" t="inlineStr">
+        <is>
+          <t>SAQ</t>
+        </is>
+      </c>
+      <c r="E3" s="9" t="inlineStr">
+        <is>
+          <t>Montréal</t>
+        </is>
+      </c>
+      <c r="F3" s="9" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="9" t="inlineStr">
+        <is>
+          <t>15544570</t>
+        </is>
+      </c>
+      <c r="B4" s="9" t="inlineStr">
+        <is>
+          <t>Beach Day Every Day Vodka Frozen Berries</t>
+        </is>
+      </c>
+      <c r="C4" s="9" t="inlineStr">
+        <is>
+          <t>Faubourg Sainte-Catherine</t>
+        </is>
+      </c>
+      <c r="D4" s="9" t="inlineStr">
+        <is>
+          <t>SAQ</t>
+        </is>
+      </c>
+      <c r="E4" s="9" t="inlineStr">
+        <is>
+          <t>Montréal</t>
+        </is>
+      </c>
+      <c r="F4" s="9" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="9" t="inlineStr">
+        <is>
+          <t>15544570</t>
+        </is>
+      </c>
+      <c r="B5" s="9" t="inlineStr">
+        <is>
+          <t>Beach Day Every Day Vodka Frozen Berries</t>
+        </is>
+      </c>
+      <c r="C5" s="9" t="inlineStr">
+        <is>
+          <t>Mont-Royal Est - Mentana</t>
+        </is>
+      </c>
+      <c r="D5" s="9" t="inlineStr">
+        <is>
+          <t>SAQ Express</t>
+        </is>
+      </c>
+      <c r="E5" s="9" t="inlineStr">
+        <is>
+          <t>Montréal</t>
+        </is>
+      </c>
+      <c r="F5" s="9" t="n">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="9" t="inlineStr">
+        <is>
+          <t>15544570</t>
+        </is>
+      </c>
+      <c r="B6" s="9" t="inlineStr">
+        <is>
+          <t>Beach Day Every Day Vodka Frozen Berries</t>
+        </is>
+      </c>
+      <c r="C6" s="9" t="inlineStr">
+        <is>
+          <t>Mont-Royal Est - Papineau</t>
+        </is>
+      </c>
+      <c r="D6" s="9" t="inlineStr">
+        <is>
+          <t>SAQ Sélection</t>
+        </is>
+      </c>
+      <c r="E6" s="9" t="inlineStr">
+        <is>
+          <t>Montréal</t>
+        </is>
+      </c>
+      <c r="F6" s="9" t="n">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="9" t="inlineStr">
+        <is>
+          <t>15544570</t>
+        </is>
+      </c>
+      <c r="B7" s="9" t="inlineStr">
+        <is>
+          <t>Beach Day Every Day Vodka Frozen Berries</t>
+        </is>
+      </c>
+      <c r="C7" s="9" t="inlineStr">
+        <is>
+          <t>Av. Laurier Est</t>
+        </is>
+      </c>
+      <c r="D7" s="9" t="inlineStr">
+        <is>
+          <t>SAQ</t>
+        </is>
+      </c>
+      <c r="E7" s="9" t="inlineStr">
+        <is>
+          <t>Montréal</t>
+        </is>
+      </c>
+      <c r="F7" s="9" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="9" t="inlineStr">
+        <is>
+          <t>15544570</t>
+        </is>
+      </c>
+      <c r="B8" s="9" t="inlineStr">
+        <is>
+          <t>Beach Day Every Day Vodka Frozen Berries</t>
+        </is>
+      </c>
+      <c r="C8" s="9" t="inlineStr">
+        <is>
+          <t>Place Longueuil</t>
+        </is>
+      </c>
+      <c r="D8" s="9" t="inlineStr">
+        <is>
+          <t>SAQ</t>
+        </is>
+      </c>
+      <c r="E8" s="9" t="inlineStr">
+        <is>
+          <t>Longueuil</t>
+        </is>
+      </c>
+      <c r="F8" s="9" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="9" t="inlineStr">
+        <is>
+          <t>15544570</t>
+        </is>
+      </c>
+      <c r="B9" s="9" t="inlineStr">
+        <is>
+          <t>Beach Day Every Day Vodka Frozen Berries</t>
+        </is>
+      </c>
+      <c r="C9" s="9" t="inlineStr">
+        <is>
+          <t>Ateliers Angus</t>
+        </is>
+      </c>
+      <c r="D9" s="9" t="inlineStr">
+        <is>
+          <t>SAQ Sélection</t>
+        </is>
+      </c>
+      <c r="E9" s="9" t="inlineStr">
+        <is>
+          <t>Montréal</t>
+        </is>
+      </c>
+      <c r="F9" s="9" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="9" t="inlineStr">
+        <is>
+          <t>15544570</t>
+        </is>
+      </c>
+      <c r="B10" s="9" t="inlineStr">
+        <is>
+          <t>Beach Day Every Day Vodka Frozen Berries</t>
+        </is>
+      </c>
+      <c r="C10" s="9" t="inlineStr">
+        <is>
+          <t>Saint-Lambert - Boul. Sir-Wilfrid-Laurier</t>
+        </is>
+      </c>
+      <c r="D10" s="9" t="inlineStr">
+        <is>
+          <t>SAQ Sélection</t>
+        </is>
+      </c>
+      <c r="E10" s="9" t="inlineStr">
+        <is>
+          <t>Saint-Lambert</t>
+        </is>
+      </c>
+      <c r="F10" s="9" t="n">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="9" t="inlineStr">
+        <is>
+          <t>15544570</t>
+        </is>
+      </c>
+      <c r="B11" s="9" t="inlineStr">
+        <is>
+          <t>Beach Day Every Day Vodka Frozen Berries</t>
+        </is>
+      </c>
+      <c r="C11" s="9" t="inlineStr">
+        <is>
+          <t>L'Île-des-Soeurs</t>
+        </is>
+      </c>
+      <c r="D11" s="9" t="inlineStr">
+        <is>
+          <t>SAQ Sélection</t>
+        </is>
+      </c>
+      <c r="E11" s="9" t="inlineStr">
+        <is>
+          <t>Montréal</t>
+        </is>
+      </c>
+      <c r="F11" s="9" t="n">
+        <v>13</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>